<commit_message>
feat: add CalledComplaints component for detailed complaint call analysis
- Implemented CalledComplaints component to display detailed information about complaints and their associated calls.
- Introduced filtering and sorting capabilities for better data management.
- Added export functionality to download complaint data as Excel files.
- Created utility functions for handling date presets and fault categorization.
- Established a canonicalization system for fault categories to ensure consistency across the application.
</commit_message>
<xml_diff>
--- a/public/DT-Count.xlsx
+++ b/public/DT-Count.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmakh\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\report\my-scraping-project\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962095CF-4019-46A8-B3CA-AE7F8241EF8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0346F13-C4E4-4CBC-9AD3-2AC8C6677EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>